<commit_message>
fix second screen bug, lat system support specify cleat tileset
</commit_message>
<xml_diff>
--- a/Supplementary/文档/Lua脚本文档.xlsx
+++ b/Supplementary/文档/Lua脚本文档.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E54AF8-825B-4EB6-B96F-297FA26AE13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E5A7E1C-D1D8-44DA-8D9F-3E8CE6B9D890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5940" yWindow="2730" windowWidth="28800" windowHeight="15370" xr2:uid="{8CA9C43F-A422-443C-91EB-82DDAA2DCA05}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1297" uniqueCount="797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1297" uniqueCount="799">
   <si>
     <t>iso_size()</t>
   </si>
@@ -12576,6 +12576,14 @@
       </rPr>
       <t>刷新覆盖物状态</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>强度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>health</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -12881,7 +12889,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -12890,10 +12898,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -17751,11 +17759,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="40" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="24" t="s">
         <v>334</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -18077,11 +18085,11 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="20" t="s">
@@ -18162,11 +18170,11 @@
       </c>
     </row>
     <row r="39" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="24" t="s">
         <v>655</v>
       </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="24"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="14" t="s">
@@ -18471,11 +18479,11 @@
       </c>
     </row>
     <row r="60" spans="1:6" ht="40" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="24" t="s">
+      <c r="A60" s="25" t="s">
         <v>657</v>
       </c>
-      <c r="B60" s="24"/>
-      <c r="C60" s="24"/>
+      <c r="B60" s="25"/>
+      <c r="C60" s="25"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="12" t="s">
@@ -19561,15 +19569,15 @@
       <c r="D146" s="1"/>
       <c r="E146" s="1"/>
     </row>
-    <row r="147" spans="1:5" ht="16" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>214</v>
+        <v>798</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>388</v>
+        <v>797</v>
       </c>
       <c r="D147" s="1"/>
       <c r="E147" s="1"/>
@@ -19582,12 +19590,12 @@
         <v>212</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D148" s="1"/>
       <c r="E148" s="1"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:5" ht="16" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>25</v>
       </c>
@@ -19595,7 +19603,7 @@
         <v>213</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D149" s="1"/>
       <c r="E149" s="1"/>
@@ -19898,11 +19906,11 @@
       <c r="E172" s="1"/>
     </row>
     <row r="173" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="21" t="s">
+      <c r="A173" s="24" t="s">
         <v>662</v>
       </c>
-      <c r="B173" s="21"/>
-      <c r="C173" s="21"/>
+      <c r="B173" s="24"/>
+      <c r="C173" s="24"/>
       <c r="D173" s="1"/>
       <c r="E173" s="1"/>
     </row>
@@ -21456,11 +21464,11 @@
       <c r="E284" s="1"/>
     </row>
     <row r="285" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A285" s="25" t="s">
+      <c r="A285" s="21" t="s">
         <v>671</v>
       </c>
-      <c r="B285" s="25"/>
-      <c r="C285" s="25"/>
+      <c r="B285" s="21"/>
+      <c r="C285" s="21"/>
       <c r="D285" s="1"/>
       <c r="E285" s="1"/>
     </row>
@@ -21842,11 +21850,11 @@
       <c r="E314" s="1"/>
     </row>
     <row r="315" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A315" s="25" t="s">
+      <c r="A315" s="21" t="s">
         <v>672</v>
       </c>
-      <c r="B315" s="25"/>
-      <c r="C315" s="25"/>
+      <c r="B315" s="21"/>
+      <c r="C315" s="21"/>
       <c r="D315" s="1"/>
       <c r="E315" s="1"/>
     </row>
@@ -22202,11 +22210,11 @@
       <c r="E342" s="1"/>
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A343" s="25" t="s">
+      <c r="A343" s="21" t="s">
         <v>673</v>
       </c>
-      <c r="B343" s="25"/>
-      <c r="C343" s="25"/>
+      <c r="B343" s="21"/>
+      <c r="C343" s="21"/>
       <c r="D343" s="1"/>
       <c r="E343" s="1"/>
     </row>
@@ -22380,11 +22388,11 @@
       <c r="E356" s="1"/>
     </row>
     <row r="357" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A357" s="25" t="s">
+      <c r="A357" s="21" t="s">
         <v>674</v>
       </c>
-      <c r="B357" s="25"/>
-      <c r="C357" s="25"/>
+      <c r="B357" s="21"/>
+      <c r="C357" s="21"/>
       <c r="D357" s="1"/>
       <c r="E357" s="1"/>
     </row>
@@ -22571,11 +22579,11 @@
       <c r="E371" s="1"/>
     </row>
     <row r="372" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A372" s="25" t="s">
+      <c r="A372" s="21" t="s">
         <v>675</v>
       </c>
-      <c r="B372" s="25"/>
-      <c r="C372" s="25"/>
+      <c r="B372" s="21"/>
+      <c r="C372" s="21"/>
       <c r="D372" s="1"/>
       <c r="E372" s="1"/>
     </row>
@@ -23201,13 +23209,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A357:C357"/>
-    <mergeCell ref="A372:C372"/>
-    <mergeCell ref="A256:C256"/>
-    <mergeCell ref="A279:C279"/>
-    <mergeCell ref="A281:C281"/>
-    <mergeCell ref="A285:C285"/>
-    <mergeCell ref="A315:C315"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A415:C415"/>
     <mergeCell ref="A121:C121"/>
@@ -23224,6 +23225,13 @@
     <mergeCell ref="A207:C207"/>
     <mergeCell ref="A230:C230"/>
     <mergeCell ref="A343:C343"/>
+    <mergeCell ref="A357:C357"/>
+    <mergeCell ref="A372:C372"/>
+    <mergeCell ref="A256:C256"/>
+    <mergeCell ref="A279:C279"/>
+    <mergeCell ref="A281:C281"/>
+    <mergeCell ref="A285:C285"/>
+    <mergeCell ref="A315:C315"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>